<commit_message>
Retoques en la paleta de colores de la tabla del excel
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,96 +458,50 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>5 de Agosto de 2026</t>
+          <t>6 de Agosto de 2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Blusas</t>
+          <t>holagff</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Envio)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5 de Agosto de 2026</t>
+          <t>6 de Agosto de 2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Envio de Paqueteria</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>17</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
+          <t>r4tr</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>344</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>-(Envio)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>5 de Agosto de 2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Pago de Renta</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>300</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>6 de Agosto de 2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>holaaa</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>37.00</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>+(Ingreso)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pequeños Cambios para hacer la interfaz mas amigable con el usuario
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,19 +489,65 @@
           <t>r4tr</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>344</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="C3" t="n">
+        <v>344</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>-(Envio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>6 de Agosto de 2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Venta Blusa Talla M</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>35</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>6 de Agosto de 2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>hoklga</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se agrego un widget que registra utilidad de Ingresos
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,19 +535,65 @@
           <t>hoklga</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="C5" t="n">
+        <v>34</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>holaa</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>34</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nosee</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>35.00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se actualizan en tiempo real los widgets de la utilidad
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -581,17 +581,132 @@
           <t>nosee</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>35.00</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="C7" t="n">
+        <v>35</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ropa de marca</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>venta de zapatoss</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>22.35</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>hola xddd</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>456</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>jhgfghgf</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>67.17</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>568</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>875.81</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>+(Ingreso)</t>
         </is>

</xml_diff>

<commit_message>
Cambios en los widgets de utilidades
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,92 +458,92 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6 de Agosto de 2026</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>holagff</t>
+          <t>Venta de Blusas Talla M</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34</v>
+        <v>34.5</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-(Envio)</t>
+          <t>+(Ingreso)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>6 de Agosto de 2026</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>r4tr</t>
+          <t>Pago de Electricidad</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>344</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-(Envio)</t>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>6 de Agosto de 2026</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Venta Blusa Talla M</t>
+          <t>Compra de Inventario</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6 de Agosto de 2026</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hoklga</t>
+          <t>gasdgsgs</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>34</v>
+        <v>3.99</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>-(Egreso)</t>
+          <t>+(Ingreso)</t>
         </is>
       </c>
     </row>
@@ -555,14 +555,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>holaa</t>
+          <t>holawatafak</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>34</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -578,18 +578,18 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>nosee</t>
+          <t>holaaa</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
         <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>
@@ -601,18 +601,18 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ropa de marca</t>
+          <t>hpolssg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7.99</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>
@@ -624,18 +624,18 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>venta de zapatoss</t>
+          <t>jhgfdfghgfd</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22.35</v>
+        <v>77</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>
@@ -647,18 +647,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hola xddd</t>
+          <t>hgddfgfdf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>456</v>
+        <v>161.85</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>
@@ -670,14 +670,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>jhgfghgf</t>
+          <t>jhgfaddfgfgfd</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>67.17</v>
+        <v>123</v>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -693,22 +693,91 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>568</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>875.81</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+          <t>hgdfgfdfgfd</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>246</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>-(Egreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>jhgfghjhgfg</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>123</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>gfdfg</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>246</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>jhghgfghgf</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>3.99</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retoques Finales de los Widgets de utilidad
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,18 +463,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Venta de Blusas Talla M</t>
+          <t>Pago Renta</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34.5</v>
+        <v>35</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+(Ingreso)</t>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>
@@ -486,298 +486,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pago de Electricidad</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>50</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
+          <t>holaaaaa</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Compra de Inventario</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>gasdgsgs</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="D5" t="n">
-        <v>15</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
           <t>+(Ingreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>holawatafak</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>34</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>+(Ingreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>holaaa</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>hpolssg</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" t="n">
-        <v>7</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>jhgfdfghgfd</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>77</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>hgddfgfdf</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>161.85</v>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>jhgfaddfgfgfd</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>123</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>+(Ingreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>hgdfgfdfgfd</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>246</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>jhgfghjhgfg</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>123</v>
-      </c>
-      <c r="D13" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>+(Ingreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>gfdfg</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>246</v>
-      </c>
-      <c r="D14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>jhghgfghgf</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>3.99</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se agregaron botones en la barra de la izquierda y el de logout funciona, aun falta arreglar la actualizacion de la fecha en tiempo real
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,19 +489,111 @@
           <t>holaaaaa</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
+      <c r="C3" t="n">
+        <v>45</v>
+      </c>
+      <c r="D3" t="n">
+        <v>67</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>+(Ingreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>jhgfdfgh</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>104.65</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-(Envio)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>jhgfdfghj</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>89.56</v>
+      </c>
+      <c r="D5" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>gfdfg</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>45.78</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>xsghgfdf</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7.00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-(Egreso)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Funciona el boton de los graficos
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -581,19 +581,42 @@
           <t>xsghgfdf</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>7.00</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>-(Egreso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>rtyuytre</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>+(Ingreso)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se arreglo un bug al cerrar la sesion que hacia que se mantenieran las utlidades del ultimo usuario
</commit_message>
<xml_diff>
--- a/Reporte-EasyFinance-Briamm.xlsx
+++ b/Reporte-EasyFinance-Briamm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,165 +458,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pago Renta</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>35</v>
-      </c>
-      <c r="D2" t="n">
-        <v>4</v>
+          <t>jasdgs</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>35.00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>holaaaaa</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>45</v>
-      </c>
-      <c r="D3" t="n">
-        <v>67</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>+(Ingreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>jhgfdfgh</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>104.65</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>-(Envio)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>jhgfdfghj</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>89.56</v>
-      </c>
-      <c r="D5" t="n">
-        <v>30</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>gfdfg</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>45.78</v>
-      </c>
-      <c r="D6" t="n">
-        <v>30</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>xsghgfdf</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>-(Egreso)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>rtyuytre</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>+(Ingreso)</t>
         </is>
       </c>
     </row>

</xml_diff>